<commit_message>
Download and content-verify all passport PDFs; curate catalog and equipment selection
- Apply per-PDF content verification (keep/relabel/remove) and round-4 research
  (fixed broken links, PPG/PPG Korea SDS, Uz-DongJu TDS, colour-matched OEM basecoats)
- Curate duplicates, superseded and wrong-class documents (round5)
- Main sheets now list only downloaded and verified PDFs; equipment comes from
  data/equipment_selection.json with official model names
- File names derived from the real document titles; downloader reuses files by URL

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XBVq9sVwo381PBpTwDGfwY
</commit_message>
<xml_diff>
--- a/output/material_equipment_names.xlsx
+++ b/output/material_equipment_names.xlsx
@@ -463,13 +463,13 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CHEMFOS 740R</t>
+          <t>CHEMFOS 740R L CLEAR</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Dürr Ecopaint RoDip</t>
+          <t>Dürr RoDip M (Ecopaint pretreatment / e-coat dip line)</t>
         </is>
       </c>
       <c r="D2" s="2" t="n"/>
@@ -483,9 +483,9 @@
       <c r="B3" s="2" t="n"/>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Dürr Ecopaint RoDip
-Controlled Power Company AACD Series 50 rectifier
-Koch Membrane Systems KPAK ultrafiltration module</t>
+          <t>Dürr RoDip M (Ecopaint pretreatment / e-coat dip line)
+Trystar Series 50 rectifier (Model 506 / 5012) with AACD controller
+Kovalus KPAK PLUS ultrafiltration module</t>
         </is>
       </c>
       <c r="D3" s="2" t="n"/>
@@ -499,9 +499,9 @@
       <c r="B4" s="2" t="n"/>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Dürr Ecopaint RoDip
-Controlled Power Company AACD Series 50 rectifier
-Koch Membrane Systems KPAK ultrafiltration module</t>
+          <t>Dürr RoDip M (Ecopaint pretreatment / e-coat dip line)
+Trystar Series 50 rectifier (Model 506 / 5012) with AACD controller
+Kovalus KPAK PLUS ultrafiltration module</t>
         </is>
       </c>
       <c r="D4" s="2" t="n"/>
@@ -515,7 +515,7 @@
       <c r="B5" s="2" t="n"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Graco E-Flo SP
+          <t>Graco E-Flo SP supply system
 Dürr EcoShot Meter
 Dürr EcoGun2 3D</t>
         </is>
@@ -531,8 +531,8 @@
       <c r="B6" s="2" t="n"/>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Graco King XL10K
-Graco AL Series Automatic Airless Spray Gun (288048)</t>
+          <t>Graco King airless pump with XL 10K air motor
+Graco AL Automatic Airless Spray Gun (288048)</t>
         </is>
       </c>
       <c r="D6" s="2" t="n"/>
@@ -546,8 +546,8 @@
       <c r="B7" s="2" t="n"/>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Graco King XL10K
-Graco AL Series Automatic Airless Spray Gun (288048)</t>
+          <t>Graco King airless pump with XL 10K air motor
+Graco AL Automatic Airless Spray Gun (288048)</t>
         </is>
       </c>
       <c r="D7" s="2" t="n"/>
@@ -561,8 +561,8 @@
       <c r="B8" s="2" t="n"/>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Graco King XL10K
-Graco AL Series Automatic Airless Spray Gun (288048)</t>
+          <t>Graco King airless pump with XL 10K air motor
+Graco AL Automatic Airless Spray Gun (288048)</t>
         </is>
       </c>
       <c r="D8" s="2" t="n"/>
@@ -807,7 +807,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>BASE TYPE THINNER</t>
+          <t>RHT-031 Top Metallic Thinner (BASE TYPE THINNER)</t>
         </is>
       </c>
       <c r="B24" s="2" t="n"/>
@@ -852,14 +852,13 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>CLEANING THINNER</t>
+          <t>RHT-031 Top Metallic Thinner (CLEANING THINNER)</t>
         </is>
       </c>
       <c r="B27" s="2" t="n"/>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Dürr EcoBell Cleaner D2
-Dürr EcoBell PurgeBox</t>
+          <t>Dürr EcoBell Cleaner D2 + EcoBell PurgeBox</t>
         </is>
       </c>
       <c r="D27" s="2" t="n"/>
@@ -867,14 +866,14 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>DISK BRAKE FLUID DOT-4 PLUS</t>
+          <t>CROWN Brake Fluid DOT-4 Plus</t>
         </is>
       </c>
       <c r="B28" s="2" t="n"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Dürr Somac ProLine Cube
-Dürr Somac G4 Blue filling adapter</t>
+Dürr Somac G4 Blue Filling Adapter</t>
         </is>
       </c>
       <c r="D28" s="2" t="n"/>
@@ -882,14 +881,14 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>POWER STRG OIL DEXRON-VI GMN10060</t>
+          <t>DEXRON-VI Power Steering Fluid (GMN10060)</t>
         </is>
       </c>
       <c r="B29" s="2" t="n"/>
       <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Dürr Somac ProLine Cube
-Dürr Somac G4 Blue filling adapter</t>
+Dürr Somac G4 Blue Filling Adapter</t>
         </is>
       </c>
       <c r="D29" s="2" t="n"/>
@@ -897,14 +896,14 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>ANTIFREEZE DX-COOL CONCENTRATE RED</t>
+          <t>ANTIFREEZE DX-COOL CONCENTRATE RED (FELIX)</t>
         </is>
       </c>
       <c r="B30" s="2" t="n"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Dürr Somac ProLine Cube
-Dürr Somac G4 Blue filling adapter</t>
+Dürr Somac G4 Blue Filling Adapter</t>
         </is>
       </c>
       <c r="D30" s="2" t="n"/>
@@ -912,13 +911,13 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>T/M OIL Idemitsu MTF LSJ11EP</t>
+          <t>Idemitsu MTF LSJ11EP</t>
         </is>
       </c>
       <c r="B31" s="2" t="n"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Dürr Somac ProLine line filling station</t>
+          <t>Dürr Somac Compact filling station</t>
         </is>
       </c>
       <c r="D31" s="2" t="n"/>
@@ -926,13 +925,13 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>T/M OIL MANUAL SH XGP 75W85 GL-4</t>
+          <t>XGP 75W-85 GL-4 Manual Transmission Fluid</t>
         </is>
       </c>
       <c r="B32" s="2" t="n"/>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Dürr Somac ProLine line filling station</t>
+          <t>Dürr Somac Compact filling station</t>
         </is>
       </c>
       <c r="D32" s="2" t="n"/>
@@ -940,13 +939,13 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>A/T OIL DEXRON-VI</t>
+          <t>DEXRON-VI Automatic Transmission Fluid</t>
         </is>
       </c>
       <c r="B33" s="2" t="n"/>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Dürr Somac ProLine line filling station</t>
+          <t>Dürr Somac Compact filling station</t>
         </is>
       </c>
       <c r="D33" s="2" t="n"/>
@@ -954,14 +953,14 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>TETRAFLUOROETHANE HFC-134a</t>
+          <t>COOLIB R134a (HFC-134a) Refrigerant</t>
         </is>
       </c>
       <c r="B34" s="2" t="n"/>
       <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Dürr Somac ProLine Cube
-Dürr Somac G4 Blue Twin A/C adapter</t>
+Dürr Somac G4 Blue Twin A/C Adapter</t>
         </is>
       </c>
       <c r="D34" s="2" t="n"/>
@@ -969,13 +968,13 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>FUEL AI-92</t>
+          <t>AI-92 Gasoline</t>
         </is>
       </c>
       <c r="B35" s="2" t="n"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Dürr Somac fuel filling station</t>
+          <t>Dürr Somac Compact Ex (fuel filling)</t>
         </is>
       </c>
       <c r="D35" s="2" t="n"/>
@@ -983,7 +982,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>WINDSHIELD WASHER (ETHANOL 80%)</t>
+          <t>Windshield Washer Fluid (Ethanol 80%)</t>
         </is>
       </c>
       <c r="B36" s="2" t="n"/>
@@ -997,14 +996,14 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>BETASEAL / SikaFlex-250 UZ-1</t>
+          <t>Sikaflex-250 UZ-1 / BETASEAL</t>
         </is>
       </c>
       <c r="B37" s="2" t="n"/>
       <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Graco Therm-O-Flow 200
-Atlas Copco SCA dispensing system</t>
+Graco PCF (Precision Continuous Flow) metering</t>
         </is>
       </c>
       <c r="D37" s="2" t="n"/>
@@ -1012,13 +1011,13 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ADHESIVE-HDLNG T/PNL</t>
+          <t>ADHESIVE-HDLNG T/PNL (headliner adhesive)</t>
         </is>
       </c>
       <c r="B38" s="2" t="n"/>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Nordson ProBlue bulk hot melt melter</t>
+          <t>Graco Therm-O-Flow 200</t>
         </is>
       </c>
       <c r="D38" s="2" t="n"/>
@@ -1026,14 +1025,14 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>RKB 0101S (SIKA-209 D)</t>
+          <t>Sika Primer-209 D</t>
         </is>
       </c>
       <c r="B39" s="2" t="n"/>
       <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Nordson EFD 752V diaphragm valve
-Graco agitated pressure tank</t>
+Graco stainless steel pressure tank with agitator</t>
         </is>
       </c>
       <c r="D39" s="2" t="n"/>
@@ -1041,14 +1040,14 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>RKB 0401S (SIKA-206 G+P)</t>
+          <t>Sika Primer-206 G+P</t>
         </is>
       </c>
       <c r="B40" s="2" t="n"/>
       <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Nordson EFD 752V diaphragm valve
-Graco agitated pressure tank</t>
+Graco stainless steel pressure tank with agitator</t>
         </is>
       </c>
       <c r="D40" s="2" t="n"/>
@@ -1056,13 +1055,13 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>BETAPRIME (100-UZ)</t>
+          <t>Sika Aktivator-100</t>
         </is>
       </c>
       <c r="B41" s="2" t="n"/>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Lint-free wipes (manual wipe-on / wipe-off)</t>
+          <t>Manual wipe-on / wipe-off (lint-free cloth)</t>
         </is>
       </c>
       <c r="D41" s="2" t="n"/>
@@ -1077,7 +1076,7 @@
       <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Nordson EFD 752V diaphragm valve
-Graco agitated pressure tank</t>
+Graco stainless steel pressure tank with agitator</t>
         </is>
       </c>
       <c r="D42" s="2" t="n"/>
@@ -1091,8 +1090,7 @@
       <c r="B43" s="2" t="n"/>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Graco Fire-Ball 300
-Lincoln PowerMaster II</t>
+          <t>Graco Fire-Ball 300 (50:1 grease pump)</t>
         </is>
       </c>
       <c r="D43" s="2" t="n"/>
@@ -1100,14 +1098,13 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>LUBRICANT-CLU PLT HUB M/T (MICROLUBE GNY-202)</t>
+          <t>Klüber MICROLUBE GNY 202</t>
         </is>
       </c>
       <c r="B44" s="2" t="n"/>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Graco Fire-Ball 300
-Lincoln PowerMaster II</t>
+          <t>Graco Fire-Ball 300 (50:1 grease pump)</t>
         </is>
       </c>
       <c r="D44" s="2" t="n"/>
@@ -1123,14 +1120,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1146,17 +1145,27 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Zavod ro'yxatidagi nomi</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Manbadagi spec</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Jihoz ishonchi</t>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Identifikatsiya ishonchi</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Jihoz (ishonch)</t>
         </is>
       </c>
     </row>
@@ -1166,22 +1175,32 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>CHEMFOS 740R</t>
+          <t>CHEMFOS 740R L CLEAR</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>CHEMFOS # 740R</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>2E+08 (Excel-truncated, full SAP unknown)</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>KR-JFR-740</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Dürr RoDip M (Ecopaint pretreatment / e-coat dip line) (medium)</t>
         </is>
       </c>
     </row>
@@ -1196,17 +1215,29 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>ED7010 Binder Gray</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>RAC07106</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>KR-E6461</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>medium</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Dürr RoDip M (Ecopaint pretreatment / e-coat dip line) (medium)
+Trystar Series 50 rectifier (Model 506 / 5012) with AACD controller (medium)
+Kovalus KPAK PLUS ultrafiltration module (medium)</t>
         </is>
       </c>
     </row>
@@ -1221,17 +1252,29 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>ED7010 Paste Gray</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>RAC07107</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>KR-E6462</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>medium</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Dürr RoDip M (Ecopaint pretreatment / e-coat dip line) (medium)
+Trystar Series 50 rectifier (Model 506 / 5012) with AACD controller (medium)
+Kovalus KPAK PLUS ultrafiltration module (medium)</t>
         </is>
       </c>
     </row>
@@ -1246,17 +1289,29 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>BODY SEALER RSB-430</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>RAC05109</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>GVH-403U</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Graco E-Flo SP supply system (medium)
+Dürr EcoShot Meter (medium)
+Dürr EcoGun2 3D (medium)</t>
         </is>
       </c>
     </row>
@@ -1271,17 +1326,28 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t>UBC UNDER COAT RSU-230</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>RAC05110</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>GVH-170</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Graco King airless pump with XL 10K air motor (medium)
+Graco AL Automatic Airless Spray Gun (288048) (medium)</t>
         </is>
       </c>
     </row>
@@ -1296,17 +1362,28 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>UBS COAT</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>RAC05137</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>GVH-170</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Graco King airless pump with XL 10K air motor (medium)
+Graco AL Automatic Airless Spray Gun (288048) (medium)</t>
         </is>
       </c>
     </row>
@@ -1321,17 +1398,28 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t>PVC ANTI CHIP</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>RAC00562</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>P8201</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Graco King airless pump with XL 10K air motor (medium)
+Graco AL Automatic Airless Spray Gun (288048) (medium)</t>
         </is>
       </c>
     </row>
@@ -1346,17 +1434,28 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>CR-100 PRIMER SURFACER LIGHT GRAY (N7.0)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
           <t>RAC07111</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>KR-APC-707U</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>medium</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)</t>
         </is>
       </c>
     </row>
@@ -1371,17 +1470,28 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>CR-100 PRIMER SURFACER PURE WHITE (N9.0)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
           <t>RAC07112</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>KR-APC-742U</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>medium</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)</t>
         </is>
       </c>
     </row>
@@ -1396,17 +1506,28 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
+          <t>PRIMER TYPE THINNER</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
           <t>RAC07113</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>KR-RHT-051</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>medium</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoSupply2 Core (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1421,17 +1542,29 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t>(GAZ) BASE COAT SUMMIT WHITE (2C1B)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
           <t>200000226</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>KR-MC-710U</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1446,17 +1579,29 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
+          <t>(GK2) BASE COAT SON OF A GUN GRAY MET-3</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
           <t>200000223</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>KR-ADM-709U</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1471,17 +1616,29 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
+          <t>(GD8) BASE COAT BURNT COCONUTMET</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
           <t>200000212</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>KR-ADM-254</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1496,17 +1653,29 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
+          <t>(GBO) BASE COAT BLACK MEET KETTLE MET-3</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
           <t>200000209</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>KR-ADM-786</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1521,17 +1690,29 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
+          <t>(GYM) BASE COAT SATIN STEEL GRAYMET</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
           <t>200000221</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>KR-ADM-706U</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1546,17 +1727,29 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
+          <t>(GAN) BASE COAT SWITCHBLADE SILVER</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
           <t>200000207</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>KR-ADM-893</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1571,17 +1764,29 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
+          <t>(GL8) BASE COAT RED-E OR NOT RED MET-3</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
           <t>200000219</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>KR-ADM-122</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1596,17 +1801,29 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
+          <t>(GUM) BASE COAT SEEKER MET 3</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
           <t>200000271</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>KR-ADM-407U</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1621,17 +1838,29 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
+          <t>(G7G) BASE COAT ZEUS</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
           <t>200002029</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>KR-ADM-670U</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1646,17 +1875,29 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
+          <t>(GZ8) BASE COAT SOME KINDA BLUE</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
           <t>200002008</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>KR-ADM-512U</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1671,17 +1912,29 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
+          <t>(G5J) BASE COAT DARKMOON BLUE</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
           <t>200001697</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>KR-ADM-513U</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1696,17 +1949,29 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
+          <t>(G4V) BASE COAT POW ZINGA MET-3</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
           <t>200001696</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>KR-ADM-580U</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1716,22 +1981,33 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
+          <t>RHT-031 Top Metallic Thinner (BASE TYPE THINNER)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
           <t>BASE TYPE THINNER</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>RAC07130</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>KR-RHT-031</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoSupply2 Core (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1746,17 +2022,28 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
+          <t>TOP CLEAR HITEC 2000</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
           <t>RAC07132</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>KR-ABT-600U</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>medium</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoRP E043i (medium)
+Dürr EcoBell3 (medium)</t>
         </is>
       </c>
     </row>
@@ -1771,17 +2058,28 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
+          <t>CLEAR THINNER</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
           <t>RAC07133</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>KR-RBT-029</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>medium</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoSupply2 Core (medium)
+Dürr EcoMCC3 20 (medium)</t>
         </is>
       </c>
     </row>
@@ -1791,22 +2089,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
+          <t>RHT-031 Top Metallic Thinner (CLEANING THINNER)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
           <t>CLEANING THINNER</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>RAC07130</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>KR-RHT-031</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Dürr EcoBell Cleaner D2 + EcoBell PurgeBox (medium)</t>
         </is>
       </c>
     </row>
@@ -1816,22 +2124,33 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>DISK BRAKE FLUID DOT-4 PLUS</t>
+          <t>CROWN Brake Fluid DOT-4 Plus</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
+          <t>DISK BRAKE FLUID DOT-4 PLUS (A/T and M/T)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
           <t>200000259</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>DOT-4+CROWN</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Dürr Somac ProLine Cube (medium)
+Dürr Somac G4 Blue Filling Adapter (medium)</t>
         </is>
       </c>
     </row>
@@ -1841,22 +2160,33 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>POWER STRG OIL DEXRON-VI GMN10060</t>
+          <t>DEXRON-VI Power Steering Fluid (GMN10060)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
+          <t>POWER STRG OIL DEXRON-VI GM N10060</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
           <t>200000261</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>GMN 10060</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Dürr Somac ProLine Cube (medium)
+Dürr Somac G4 Blue Filling Adapter (medium)</t>
         </is>
       </c>
     </row>
@@ -1866,22 +2196,33 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
+          <t>ANTIFREEZE DX-COOL CONCENTRATE RED (FELIX)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
           <t>ANTIFREEZE DX-COOL CONCENTRATE RED</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>200000265</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Felix</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>medium</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Dürr Somac ProLine Cube (medium)
+Dürr Somac G4 Blue Filling Adapter (medium)</t>
         </is>
       </c>
     </row>
@@ -1891,22 +2232,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>T/M OIL Idemitsu MTF LSJ11EP</t>
+          <t>Idemitsu MTF LSJ11EP</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
+          <t>T/M OIL</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
           <t>100129935</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Idemitsu MTF LSJ11EP</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Dürr Somac Compact filling station (low)</t>
         </is>
       </c>
     </row>
@@ -1916,22 +2267,32 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
+          <t>XGP 75W-85 GL-4 Manual Transmission Fluid</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
           <t>T/M OIL MANUAL SH XGP 75W85 GL-4</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>200000249</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>API GL-4</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Dürr Somac Compact filling station (low)</t>
         </is>
       </c>
     </row>
@@ -1941,22 +2302,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
+          <t>DEXRON-VI Automatic Transmission Fluid</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
           <t>A/T OIL DEXRON-VI</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>200000262</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>GMN 10060</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>low</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Dürr Somac Compact filling station (low)</t>
         </is>
       </c>
     </row>
@@ -1966,22 +2337,33 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
+          <t>COOLIB R134a (HFC-134a) Refrigerant</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
           <t>TETRAFLUOROETHANE HFC-134a</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>200000266</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>COOLIB</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>medium</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Dürr Somac ProLine Cube (medium)
+Dürr Somac G4 Blue Twin A/C Adapter (medium)</t>
         </is>
       </c>
     </row>
@@ -1991,22 +2373,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>FUEL AI-92</t>
+          <t>AI-92 Gasoline</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
+          <t>FUEL</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>AI-92</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Dürr Somac Compact Ex (fuel filling) (low)</t>
         </is>
       </c>
     </row>
@@ -2016,22 +2408,32 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>WINDSHIELD WASHER (ETHANOL 80%)</t>
+          <t>Windshield Washer Fluid (Ethanol 80%)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
+          <t>WINDSHIELD WASHER (ETHANOL - 80%)</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
           <t>200000252</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Dürr Somac ProLine Cube (medium)</t>
         </is>
       </c>
     </row>
@@ -2041,22 +2443,33 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
+          <t>Sikaflex-250 UZ-1 / BETASEAL</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
           <t>BETASEAL / SikaFlex-250 UZ-1</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>200000267</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>ADHESIVE-W/S</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>medium</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Graco Therm-O-Flow 200 (medium)
+Graco PCF (Precision Continuous Flow) metering (medium)</t>
         </is>
       </c>
     </row>
@@ -2066,22 +2479,32 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
+          <t>ADHESIVE-HDLNG T/PNL (headliner adhesive)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
           <t>ADHESIVE-HDLNG T/PNL</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>low</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Graco Therm-O-Flow 200 (medium)</t>
         </is>
       </c>
     </row>
@@ -2091,22 +2514,33 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>RKB 0101S (SIKA-209 D)</t>
+          <t>Sika Primer-209 D</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
+          <t>RKB 0101S</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
           <t>100057936</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>SIKA-209 D</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Nordson EFD 752V diaphragm valve (low)
+Graco stainless steel pressure tank with agitator (low)</t>
         </is>
       </c>
     </row>
@@ -2116,22 +2550,33 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>RKB 0401S (SIKA-206 G+P)</t>
+          <t>Sika Primer-206 G+P</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
+          <t>RKB 0401S</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
           <t>100057937</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>SIKA-206 G+P</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Nordson EFD 752V diaphragm valve (low)
+Graco stainless steel pressure tank with agitator (low)</t>
         </is>
       </c>
     </row>
@@ -2141,22 +2586,32 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>BETAPRIME (100-UZ)</t>
+          <t>Sika Aktivator-100</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
+          <t>BETAPRIME</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>100 - UZ</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>medium</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Manual wipe-on / wipe-off (lint-free cloth) (medium)</t>
         </is>
       </c>
     </row>
@@ -2171,17 +2626,28 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
+          <t>RAD 11724</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>SIKA - 100 - UZ</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>low</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Nordson EFD 752V diaphragm valve (low)
+Graco stainless steel pressure tank with agitator (low)</t>
         </is>
       </c>
     </row>
@@ -2196,17 +2662,27 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
+          <t>LUBRICANT-WHL PILOT HOLE</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>low</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Graco Fire-Ball 300 (50:1 grease pump) (low)</t>
         </is>
       </c>
     </row>
@@ -2216,22 +2692,32 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>LUBRICANT-CLU PLT HUB M/T (MICROLUBE GNY-202)</t>
+          <t>Klüber MICROLUBE GNY 202</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
+          <t>LUBRICANT-CLU PLT HUB M/T</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>MICROLUBE GNY-202</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Graco Fire-Ball 300 (50:1 grease pump) (low)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply final review fixes
- RAD 11724: drop unverified Aktivator-100 match (plant lists it as paint)
- Remove hypoid axle SDS (XGP), AGRSS training worksheet (glazing)
- Identity-evidence docs and papers no longer shown as passports
- PVC underbody/anti-chip: Henkel TEROSON PV 3046 plastisol TDS as equivalent
- Headliner hot-melt: Graco InvisiPac HM25/HM50 (pellet feed from bulk box)
- Show 'no public PDF' per undocumented equipment; Somac doc notes and
  official Dürr product pages as evidence
- Manbalar lists every shown equipment passport; factual notes only
- Names: cleaning thinner and PS fluid names; source spelling notes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XBVq9sVwo381PBpTwDGfwY
</commit_message>
<xml_diff>
--- a/output/material_equipment_names.xlsx
+++ b/output/material_equipment_names.xlsx
@@ -852,7 +852,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>RHT-031 Top Metallic Thinner (CLEANING THINNER)</t>
+          <t>CLEANING THINNER (KR-RHT-031)</t>
         </is>
       </c>
       <c r="B27" s="2" t="n"/>
@@ -881,7 +881,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>DEXRON-VI Power Steering Fluid (GMN10060)</t>
+          <t>POWER STRG OIL DEXRON-VI (GMN10060)</t>
         </is>
       </c>
       <c r="B29" s="2" t="n"/>
@@ -1017,7 +1017,7 @@
       <c r="B38" s="2" t="n"/>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Graco Therm-O-Flow 200</t>
+          <t>Graco InvisiPac HM25 / HM50 Tank-Free hot melt system</t>
         </is>
       </c>
       <c r="D38" s="2" t="n"/>
@@ -2089,7 +2089,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>RHT-031 Top Metallic Thinner (CLEANING THINNER)</t>
+          <t>CLEANING THINNER (KR-RHT-031)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>DEXRON-VI Power Steering Fluid (GMN10060)</t>
+          <t>POWER STRG OIL DEXRON-VI (GMN10060)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Graco Therm-O-Flow 200 (medium)</t>
+          <t>Graco InvisiPac HM25 / HM50 Tank-Free hot melt system (low)</t>
         </is>
       </c>
     </row>

</xml_diff>